<commit_message>
updated code for baseline
</commit_message>
<xml_diff>
--- a/docs/thesis/trial_results.xlsx
+++ b/docs/thesis/trial_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\embedded-gauge-reading-tinyml\docs\thesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D63BF7E-C852-4430-9B41-5F34AAC07EC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDE70EB8-9165-4204-B910-1993A21842E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="28110" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="27870" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,6 +35,28 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
@@ -53,13 +75,13 @@
     <t>CNN Error (°C)</t>
   </si>
   <si>
-    <t>Ideal Conditions (camera 20cm from  gauge face, bright 60 lux room, no occlusion etc.)</t>
-  </si>
-  <si>
     <t>Date Taken</t>
   </si>
   <si>
     <t>Trial #</t>
+  </si>
+  <si>
+    <t>Ideal Conditions (camera 15cm from  gauge face, bright 62 lux room, no occlusion, dirt etc. on the gauge)</t>
   </si>
 </sst>
 </file>
@@ -95,12 +117,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -126,8 +149,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EA761F53-6EB9-430F-AD0B-641F58B9F8E6}" name="Table1" displayName="Table1" ref="A2:G13" totalsRowShown="0">
-  <autoFilter ref="A2:G13" xr:uid="{EA761F53-6EB9-430F-AD0B-641F58B9F8E6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EA761F53-6EB9-430F-AD0B-641F58B9F8E6}" name="Table1" displayName="Table1" ref="A2:G14" totalsRowShown="0">
+  <autoFilter ref="A2:G14" xr:uid="{EA761F53-6EB9-430F-AD0B-641F58B9F8E6}"/>
   <tableColumns count="7">
     <tableColumn id="6" xr3:uid="{D4C4D1C6-7F44-49E2-B9C5-12F2F88B04E7}" name="Date Taken"/>
     <tableColumn id="7" xr3:uid="{5263C883-55CF-4106-ABC4-D540FDA7BCC2}" name="Trial #"/>
@@ -408,7 +431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.6640625" customWidth="1"/>
@@ -422,7 +445,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -431,10 +454,10 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
         <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
       </c>
       <c r="C2" t="s">
         <v>0</v>
@@ -463,18 +486,18 @@
         <v>-30</v>
       </c>
       <c r="D3">
-        <v>-23.3</v>
+        <v>-26.1</v>
       </c>
       <c r="E3">
         <f t="shared" ref="E3:E13" si="0">C3-D3</f>
-        <v>-6.6999999999999993</v>
+        <v>-3.8999999999999986</v>
       </c>
       <c r="F3">
-        <v>-28.4</v>
+        <v>-27</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G13" si="1">C3-F3</f>
-        <v>-1.6000000000000014</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -487,13 +510,19 @@
       <c r="C4">
         <v>-20</v>
       </c>
+      <c r="D4">
+        <v>-18.3</v>
+      </c>
       <c r="E4">
-        <f t="shared" si="0"/>
-        <v>-20</v>
+        <f>C4-F4</f>
+        <v>2.1999999999999993</v>
+      </c>
+      <c r="F4">
+        <v>-22.2</v>
       </c>
       <c r="G4">
-        <f t="shared" si="1"/>
-        <v>-20</v>
+        <f>C4-F4</f>
+        <v>2.1999999999999993</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -506,13 +535,19 @@
       <c r="C5">
         <v>-15</v>
       </c>
+      <c r="D5">
+        <v>-14.9</v>
+      </c>
       <c r="E5">
         <f t="shared" si="0"/>
-        <v>-15</v>
+        <v>-9.9999999999999645E-2</v>
+      </c>
+      <c r="F5">
+        <v>-13.2</v>
       </c>
       <c r="G5">
         <f t="shared" si="1"/>
-        <v>-15</v>
+        <v>-1.8000000000000007</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -525,13 +560,19 @@
       <c r="C6">
         <v>-5</v>
       </c>
+      <c r="D6">
+        <v>-7.3</v>
+      </c>
       <c r="E6">
         <f t="shared" si="0"/>
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="F6">
         <v>-5</v>
       </c>
       <c r="G6">
         <f t="shared" si="1"/>
-        <v>-5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -544,13 +585,19 @@
       <c r="C7">
         <v>0</v>
       </c>
+      <c r="D7">
+        <v>-0.1</v>
+      </c>
       <c r="E7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.1</v>
+      </c>
+      <c r="F7">
+        <v>1.2</v>
       </c>
       <c r="G7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -563,13 +610,19 @@
       <c r="C8">
         <v>10</v>
       </c>
+      <c r="D8">
+        <v>9.3000000000000007</v>
+      </c>
       <c r="E8">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>0.69999999999999929</v>
+      </c>
+      <c r="F8">
+        <v>7.6</v>
       </c>
       <c r="G8">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>2.4000000000000004</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -582,13 +635,19 @@
       <c r="C9">
         <v>15</v>
       </c>
+      <c r="D9">
+        <v>36.4</v>
+      </c>
       <c r="E9">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>-21.4</v>
+      </c>
+      <c r="F9">
+        <v>16.100000000000001</v>
       </c>
       <c r="G9">
         <f t="shared" si="1"/>
-        <v>15</v>
+        <v>-1.1000000000000014</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -601,13 +660,19 @@
       <c r="C10">
         <v>25</v>
       </c>
+      <c r="D10">
+        <v>32.9</v>
+      </c>
       <c r="E10">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>-7.8999999999999986</v>
+      </c>
+      <c r="F10">
+        <v>27.4</v>
       </c>
       <c r="G10">
         <f t="shared" si="1"/>
-        <v>25</v>
+        <v>-2.3999999999999986</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -620,13 +685,19 @@
       <c r="C11">
         <v>30</v>
       </c>
+      <c r="D11">
+        <v>38.799999999999997</v>
+      </c>
       <c r="E11">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>-8.7999999999999972</v>
+      </c>
+      <c r="F11">
+        <v>33.299999999999997</v>
       </c>
       <c r="G11">
         <f t="shared" si="1"/>
-        <v>30</v>
+        <v>-3.2999999999999972</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -639,13 +710,19 @@
       <c r="C12">
         <v>40</v>
       </c>
+      <c r="D12">
+        <v>33.299999999999997</v>
+      </c>
       <c r="E12">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>6.7000000000000028</v>
+      </c>
+      <c r="F12">
+        <v>34.5</v>
       </c>
       <c r="G12">
         <f t="shared" si="1"/>
-        <v>40</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -658,13 +735,31 @@
       <c r="C13">
         <v>50</v>
       </c>
+      <c r="D13">
+        <v>-16</v>
+      </c>
       <c r="E13">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>66</v>
+      </c>
+      <c r="F13">
+        <v>46.4</v>
       </c>
       <c r="G13">
         <f t="shared" si="1"/>
-        <v>50</v>
+        <v>3.6000000000000014</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="2"/>
+      <c r="E14" s="3" cm="1">
+        <f t="array" ref="E14">SUM(ABS(E3:E13))</f>
+        <v>120.1</v>
+      </c>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3" cm="1">
+        <f t="array" ref="G14">SUM(ABS(G3:G13))</f>
+        <v>26.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: sync diagrams and thesis references
</commit_message>
<xml_diff>
--- a/docs/thesis/trial_results.xlsx
+++ b/docs/thesis/trial_results.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\embedded-gauge-reading-tinyml\docs\thesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A704468-5536-453C-B471-73FC93D14161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F07EA728-B3CA-4D21-8745-C5BD7A9E7759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-13155" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Littlegood Temp Gauge" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -119,11 +119,11 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent2" xfId="1" builtinId="34"/>
@@ -452,13 +452,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
@@ -473,13 +473,13 @@
       <c r="D2" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>2</v>
       </c>
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
@@ -771,14 +771,14 @@
       <c r="D14">
         <v>-28.2</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E14" s="3">
         <f t="shared" si="0"/>
         <v>-1.8000000000000007</v>
       </c>
       <c r="F14">
         <v>-28.5</v>
       </c>
-      <c r="G14" s="3">
+      <c r="G14" s="2">
         <f t="shared" si="1"/>
         <v>-1.5</v>
       </c>
@@ -796,14 +796,14 @@
       <c r="D15">
         <v>-22.3</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="3">
         <f t="shared" si="0"/>
         <v>2.3000000000000007</v>
       </c>
       <c r="F15">
         <v>-19.5</v>
       </c>
-      <c r="G15" s="3">
+      <c r="G15" s="2">
         <f t="shared" si="1"/>
         <v>-0.5</v>
       </c>
@@ -821,14 +821,14 @@
       <c r="D16">
         <v>-21.3</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="3">
         <f t="shared" si="0"/>
         <v>6.3000000000000007</v>
       </c>
       <c r="F16">
         <v>-15.9</v>
       </c>
-      <c r="G16" s="3">
+      <c r="G16" s="2">
         <f t="shared" si="1"/>
         <v>0.90000000000000036</v>
       </c>
@@ -846,14 +846,14 @@
       <c r="D17">
         <v>-28</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="3">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="F17">
         <v>-5.2</v>
       </c>
-      <c r="G17" s="3">
+      <c r="G17" s="2">
         <f t="shared" si="1"/>
         <v>0.20000000000000018</v>
       </c>
@@ -871,14 +871,14 @@
       <c r="D18">
         <v>-29.8</v>
       </c>
-      <c r="E18" s="4">
+      <c r="E18" s="3">
         <f t="shared" si="0"/>
         <v>29.8</v>
       </c>
       <c r="F18">
         <v>-2.2000000000000002</v>
       </c>
-      <c r="G18" s="3">
+      <c r="G18" s="2">
         <f t="shared" si="1"/>
         <v>2.2000000000000002</v>
       </c>
@@ -896,14 +896,14 @@
       <c r="D19">
         <v>12</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="3">
         <f t="shared" si="0"/>
         <v>-2</v>
       </c>
       <c r="F19">
         <v>9.8000000000000007</v>
       </c>
-      <c r="G19" s="3">
+      <c r="G19" s="2">
         <f t="shared" si="1"/>
         <v>0.19999999999999929</v>
       </c>
@@ -921,14 +921,14 @@
       <c r="D20">
         <v>-22</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E20" s="3">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
       <c r="F20">
         <v>16</v>
       </c>
-      <c r="G20" s="3">
+      <c r="G20" s="2">
         <f t="shared" si="1"/>
         <v>-1</v>
       </c>
@@ -946,14 +946,14 @@
       <c r="D21">
         <v>-29</v>
       </c>
-      <c r="E21" s="4">
+      <c r="E21" s="3">
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
       <c r="F21">
         <v>28.1</v>
       </c>
-      <c r="G21" s="3">
+      <c r="G21" s="2">
         <f t="shared" si="1"/>
         <v>-3.1000000000000014</v>
       </c>
@@ -971,14 +971,14 @@
       <c r="D22">
         <v>-29</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E22" s="3">
         <f t="shared" si="0"/>
         <v>59</v>
       </c>
       <c r="F22">
         <v>32.200000000000003</v>
       </c>
-      <c r="G22" s="3">
+      <c r="G22" s="2">
         <f t="shared" si="1"/>
         <v>-2.2000000000000028</v>
       </c>
@@ -996,14 +996,14 @@
       <c r="D23">
         <v>-25.9</v>
       </c>
-      <c r="E23" s="4">
+      <c r="E23" s="3">
         <f t="shared" si="0"/>
         <v>65.900000000000006</v>
       </c>
       <c r="F23">
         <v>39.9</v>
       </c>
-      <c r="G23" s="3">
+      <c r="G23" s="2">
         <f t="shared" si="1"/>
         <v>0.10000000000000142</v>
       </c>
@@ -1021,14 +1021,14 @@
       <c r="D24">
         <v>-10.5</v>
       </c>
-      <c r="E24" s="4">
+      <c r="E24" s="3">
         <f t="shared" si="0"/>
         <v>60.5</v>
       </c>
       <c r="F24">
         <v>52.2</v>
       </c>
-      <c r="G24" s="3">
+      <c r="G24" s="2">
         <f t="shared" si="1"/>
         <v>-2.2000000000000028</v>
       </c>

</xml_diff>